<commit_message>
Pxy of remaining mixtures
</commit_message>
<xml_diff>
--- a/Experimental_data/Impurities.xlsx
+++ b/Experimental_data/Impurities.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\darshanraju\OneDrive - Delft University of Technology\Desktop\A6\Experimental_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C506C6A-CED6-452E-BA93-04E6595702BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0EAD86F-651B-41E6-9495-898EEFE91BDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PCP-SAFT" sheetId="1" r:id="rId1"/>
@@ -285,7 +285,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -319,6 +319,21 @@
       <u/>
       <sz val="12"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -622,7 +637,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -636,7 +651,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -661,7 +675,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -671,6 +684,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3139,10 +3161,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="15" t="s">
         <v>6</v>
       </c>
       <c r="C1" s="10" t="s">
@@ -3163,21 +3185,21 @@
       <c r="H1" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="J1" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="K1" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="L1" s="14" t="s">
+      <c r="L1" s="13" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="7"/>
@@ -3187,19 +3209,19 @@
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="36" t="s">
         <v>80</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="36" t="s">
         <v>80</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="36" t="s">
         <v>80</v>
       </c>
       <c r="L2" s="5"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="9"/>
@@ -3207,61 +3229,61 @@
       <c r="D3" s="6"/>
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
-      <c r="G3" s="15">
+      <c r="G3" s="14">
         <v>0</v>
       </c>
       <c r="H3" s="5"/>
-      <c r="I3" s="32">
+      <c r="I3" s="37">
         <v>0</v>
       </c>
-      <c r="J3" s="32">
+      <c r="J3" s="37">
         <v>0</v>
       </c>
-      <c r="K3" s="32">
+      <c r="K3" s="37">
         <v>0</v>
       </c>
       <c r="L3" s="6"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="21"/>
+      <c r="C4" s="20"/>
       <c r="D4" s="4"/>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
-      <c r="I4" s="15">
+      <c r="I4" s="38">
         <v>0</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="36" t="s">
         <v>80</v>
       </c>
-      <c r="K4" s="15">
+      <c r="K4" s="38">
         <v>0</v>
       </c>
-      <c r="L4" s="15">
+      <c r="L4" s="14">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="21"/>
+      <c r="C5" s="20"/>
       <c r="D5" s="8"/>
       <c r="E5" s="7"/>
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
-      <c r="I5" s="15">
+      <c r="I5" s="38">
         <v>0</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="J5" s="36" t="s">
         <v>80</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="K5" s="36" t="s">
         <v>80</v>
       </c>
       <c r="L5" s="3" t="s">
@@ -3269,23 +3291,23 @@
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="21"/>
+      <c r="C6" s="20"/>
       <c r="E6" s="8"/>
       <c r="F6" s="7"/>
-      <c r="G6" s="15">
+      <c r="G6" s="14">
         <v>0</v>
       </c>
       <c r="H6" s="5"/>
-      <c r="I6" s="15">
+      <c r="I6" s="38">
         <v>0</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="36" t="s">
         <v>80</v>
       </c>
-      <c r="K6" s="3">
+      <c r="K6" s="36">
         <v>0</v>
       </c>
       <c r="L6" s="3" t="s">
@@ -3293,164 +3315,182 @@
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="21"/>
+      <c r="C7" s="20"/>
       <c r="F7" s="8"/>
       <c r="G7" s="4"/>
-      <c r="H7" s="15">
+      <c r="H7" s="14">
         <v>0</v>
       </c>
-      <c r="I7" s="15">
+      <c r="I7" s="38">
         <v>0</v>
       </c>
-      <c r="J7" s="15">
+      <c r="J7" s="38">
         <v>0</v>
       </c>
-      <c r="K7" s="3" t="s">
+      <c r="K7" s="36" t="s">
         <v>80</v>
       </c>
-      <c r="L7" s="15">
+      <c r="L7" s="14">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="21"/>
+      <c r="C8" s="20"/>
       <c r="H8" s="7"/>
-      <c r="I8" s="15">
+      <c r="I8" s="38">
         <v>0</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="J8" s="36" t="s">
         <v>80</v>
       </c>
-      <c r="K8" s="3"/>
+      <c r="K8" s="36"/>
       <c r="L8" s="3" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="19" t="s">
         <v>24</v>
       </c>
       <c r="H9" s="8"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="15">
+      <c r="I9" s="39"/>
+      <c r="J9" s="38">
         <v>0</v>
       </c>
-      <c r="K9" s="15">
+      <c r="K9" s="38">
         <v>0</v>
       </c>
-      <c r="L9" s="15">
+      <c r="L9" s="14">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="I10" s="8"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="15" t="s">
+      <c r="I10" s="40"/>
+      <c r="J10" s="41"/>
+      <c r="K10" s="38" t="s">
         <v>80</v>
       </c>
-      <c r="L10" s="15">
+      <c r="L10" s="14">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="J11" s="8"/>
-      <c r="K11" s="4"/>
-      <c r="L11" s="15">
+      <c r="I11" s="42"/>
+      <c r="J11" s="40"/>
+      <c r="K11" s="41"/>
+      <c r="L11" s="14">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="20" t="s">
+      <c r="A12" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="K12" s="8"/>
+      <c r="I12" s="42"/>
+      <c r="J12" s="42"/>
+      <c r="K12" s="40"/>
       <c r="L12" s="4"/>
     </row>
-    <row r="14" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I13" s="42"/>
+      <c r="J13" s="42"/>
+      <c r="K13" s="42"/>
+    </row>
+    <row r="14" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I14" s="42"/>
+      <c r="J14" s="42"/>
+      <c r="K14" s="42"/>
+    </row>
     <row r="15" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D15" s="26"/>
-      <c r="E15" s="33" t="s">
+      <c r="D15" s="25"/>
+      <c r="E15" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="34"/>
-      <c r="G15" s="35"/>
+      <c r="F15" s="32"/>
+      <c r="G15" s="33"/>
+      <c r="I15" s="42"/>
+      <c r="J15" s="42"/>
+      <c r="K15" s="42"/>
     </row>
     <row r="16" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D16" s="27"/>
-      <c r="E16" s="33" t="s">
+      <c r="D16" s="26"/>
+      <c r="E16" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="F16" s="34"/>
-      <c r="G16" s="35"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="33"/>
+      <c r="I16" s="42"/>
+      <c r="J16" s="42"/>
+      <c r="K16" s="42"/>
     </row>
     <row r="17" spans="4:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D17" s="28"/>
-      <c r="E17" s="33" t="s">
+      <c r="D17" s="27"/>
+      <c r="E17" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="F17" s="34"/>
-      <c r="G17" s="35"/>
+      <c r="F17" s="32"/>
+      <c r="G17" s="33"/>
     </row>
     <row r="18" spans="4:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D18" s="25"/>
-      <c r="E18" s="33" t="s">
+      <c r="D18" s="24"/>
+      <c r="E18" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="F18" s="34"/>
-      <c r="G18" s="35"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="33"/>
     </row>
     <row r="19" spans="4:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D19" s="25"/>
-      <c r="E19" s="33" t="s">
+      <c r="D19" s="24"/>
+      <c r="E19" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="F19" s="34"/>
-      <c r="G19" s="35"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="33"/>
     </row>
     <row r="20" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R20" s="23"/>
+      <c r="R20" s="22"/>
     </row>
     <row r="21" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R21" s="24"/>
+      <c r="R21" s="23"/>
     </row>
     <row r="22" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R22" s="24"/>
+      <c r="R22" s="23"/>
     </row>
     <row r="23" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R23" s="24"/>
+      <c r="R23" s="23"/>
     </row>
     <row r="24" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R24" s="24"/>
+      <c r="R24" s="23"/>
     </row>
     <row r="25" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R25" s="24"/>
+      <c r="R25" s="23"/>
     </row>
     <row r="26" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R26" s="24"/>
+      <c r="R26" s="23"/>
     </row>
     <row r="27" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R27" s="24"/>
+      <c r="R27" s="23"/>
     </row>
     <row r="28" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R28" s="24"/>
+      <c r="R28" s="23"/>
     </row>
     <row r="29" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R29" s="24"/>
+      <c r="R29" s="23"/>
     </row>
     <row r="30" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R30" s="24"/>
+      <c r="R30" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3497,7 +3537,7 @@
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="21" t="s">
         <v>38</v>
       </c>
     </row>
@@ -3667,7 +3707,7 @@
       <c r="D9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="30">
+      <c r="E9" s="29">
         <v>2148878</v>
       </c>
     </row>
@@ -3735,7 +3775,7 @@
       <c r="D13" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="31" t="s">
+      <c r="E13" s="30" t="s">
         <v>78</v>
       </c>
     </row>
@@ -3798,7 +3838,7 @@
       <c r="E17" s="3"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="H18" s="29"/>
+      <c r="H18" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update H2S binary pairs: rename folders to underscore convention, add CO_H2S/H2_H2S results, fix N2_H2S notebook
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Experimental_data/Impurities.xlsx
+++ b/Experimental_data/Impurities.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\darshanraju\OneDrive - Delft University of Technology\Desktop\A6\Experimental_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0EAD86F-651B-41E6-9495-898EEFE91BDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A03B692C-1F15-47FE-AF37-A7AC01320820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="81">
   <si>
     <t>Molecules</t>
   </si>
@@ -285,7 +285,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -338,8 +338,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -382,6 +389,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="20">
     <border>
@@ -637,7 +650,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -675,6 +688,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -684,15 +706,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1965,6 +1979,136 @@
     </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>196453</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>41672</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>321469</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>147207</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId23">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="20" name="Ink 19">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{420F67C1-5F43-4FFB-964A-B96EDFA14D1E}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="7090172" y="1464469"/>
+            <a:ext cx="125016" cy="105535"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback xmlns="">
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="10" name="Ink 9">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5225B6B6-C1CD-4675-B722-79F91E20B070}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="5717925" y="264870"/>
+              <a:ext cx="142619" cy="123124"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>125016</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>53577</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>250032</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>159112</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId24">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="23" name="Ink 22">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8AAD583A-2E58-4914-8895-6A7BB3F3E8CF}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="7018735" y="464343"/>
+            <a:ext cx="125016" cy="105535"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback xmlns="">
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="10" name="Ink 9">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5225B6B6-C1CD-4675-B722-79F91E20B070}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="5717925" y="264870"/>
+              <a:ext cx="142619" cy="123124"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2309,6 +2453,60 @@
         </inkml:channelProperties>
       </inkml:inkSource>
       <inkml:timestamp xml:id="ts0" timeString="2026-04-20T14:50:21.414"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 232 24575,'14'14'0,"-6"-5"0,1 0 0,10 7 0,-15-13 0,-3-1 0,1-1 0,0 0 0,0 1 0,0-1 0,4 1 0,-5-1 0,-1-1 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0-1 0,-1 1 0,1 0 0,-1 0 0,1-1 0,-1 1 0,1 0 0,0-1 0,-1 1 0,1-1 0,-1 1 0,1-1 0,4-5 0,5-8 0,3-3 0,53-52 0,10-13 0,-51 52-682,38-35-1,-59 60-6143</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink21.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-04-22T13:26:52.595"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 232 24575,'14'14'0,"-6"-5"0,1 0 0,10 7 0,-15-13 0,-3-1 0,1-1 0,0 0 0,0 1 0,0-1 0,4 1 0,-5-1 0,-1-1 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0-1 0,-1 1 0,1 0 0,-1 0 0,1-1 0,-1 1 0,1 0 0,0-1 0,-1 1 0,1-1 0,-1 1 0,1-1 0,4-5 0,5-8 0,3-3 0,53-52 0,10-13 0,-51 52-682,38-35-1,-59 60-6143</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink22.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-04-22T13:39:09.406"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
       <inkml:brushProperty name="width" value="0.05" units="cm"/>
@@ -3185,13 +3383,13 @@
       <c r="H1" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="34" t="s">
+      <c r="I1" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="35" t="s">
+      <c r="J1" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="K1" s="35" t="s">
+      <c r="K1" s="32" t="s">
         <v>27</v>
       </c>
       <c r="L1" s="13" t="s">
@@ -3209,13 +3407,13 @@
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
-      <c r="I2" s="36" t="s">
+      <c r="I2" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="J2" s="36" t="s">
+      <c r="J2" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="K2" s="36" t="s">
+      <c r="K2" s="33" t="s">
         <v>80</v>
       </c>
       <c r="L2" s="5"/>
@@ -3233,13 +3431,13 @@
         <v>0</v>
       </c>
       <c r="H3" s="5"/>
-      <c r="I3" s="37">
+      <c r="I3" s="34">
         <v>0</v>
       </c>
-      <c r="J3" s="37">
+      <c r="J3" s="34">
         <v>0</v>
       </c>
-      <c r="K3" s="37">
+      <c r="K3" s="34">
         <v>0</v>
       </c>
       <c r="L3" s="6"/>
@@ -3254,13 +3452,13 @@
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
-      <c r="I4" s="38">
+      <c r="I4" s="35">
         <v>0</v>
       </c>
-      <c r="J4" s="36" t="s">
+      <c r="J4" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="K4" s="38">
+      <c r="K4" s="35">
         <v>0</v>
       </c>
       <c r="L4" s="14">
@@ -3277,13 +3475,13 @@
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
-      <c r="I5" s="38">
+      <c r="I5" s="35">
         <v>0</v>
       </c>
-      <c r="J5" s="36" t="s">
+      <c r="J5" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="K5" s="36" t="s">
+      <c r="K5" s="33" t="s">
         <v>80</v>
       </c>
       <c r="L5" s="3" t="s">
@@ -3301,13 +3499,13 @@
         <v>0</v>
       </c>
       <c r="H6" s="5"/>
-      <c r="I6" s="38">
+      <c r="I6" s="35">
         <v>0</v>
       </c>
-      <c r="J6" s="36" t="s">
+      <c r="J6" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="K6" s="36">
+      <c r="K6" s="33">
         <v>0</v>
       </c>
       <c r="L6" s="3" t="s">
@@ -3324,13 +3522,13 @@
       <c r="H7" s="14">
         <v>0</v>
       </c>
-      <c r="I7" s="38">
+      <c r="I7" s="35">
         <v>0</v>
       </c>
-      <c r="J7" s="38">
+      <c r="J7" s="35">
         <v>0</v>
       </c>
-      <c r="K7" s="36" t="s">
+      <c r="K7" s="33" t="s">
         <v>80</v>
       </c>
       <c r="L7" s="14">
@@ -3343,27 +3541,25 @@
       </c>
       <c r="C8" s="20"/>
       <c r="H8" s="7"/>
-      <c r="I8" s="38">
+      <c r="I8" s="35">
         <v>0</v>
       </c>
-      <c r="J8" s="36" t="s">
+      <c r="J8" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="K8" s="36"/>
-      <c r="L8" s="3" t="s">
-        <v>80</v>
-      </c>
+      <c r="K8" s="33"/>
+      <c r="L8" s="43"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>24</v>
       </c>
       <c r="H9" s="8"/>
-      <c r="I9" s="39"/>
-      <c r="J9" s="38">
+      <c r="I9" s="36"/>
+      <c r="J9" s="35">
         <v>0</v>
       </c>
-      <c r="K9" s="38">
+      <c r="K9" s="35">
         <v>0</v>
       </c>
       <c r="L9" s="14">
@@ -3374,9 +3570,9 @@
       <c r="A10" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="I10" s="40"/>
-      <c r="J10" s="41"/>
-      <c r="K10" s="38" t="s">
+      <c r="I10" s="37"/>
+      <c r="J10" s="38"/>
+      <c r="K10" s="35" t="s">
         <v>80</v>
       </c>
       <c r="L10" s="14">
@@ -3387,9 +3583,9 @@
       <c r="A11" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="I11" s="42"/>
-      <c r="J11" s="40"/>
-      <c r="K11" s="41"/>
+      <c r="I11" s="39"/>
+      <c r="J11" s="37"/>
+      <c r="K11" s="38"/>
       <c r="L11" s="14">
         <v>0</v>
       </c>
@@ -3398,66 +3594,66 @@
       <c r="A12" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="42"/>
-      <c r="J12" s="42"/>
-      <c r="K12" s="40"/>
+      <c r="I12" s="39"/>
+      <c r="J12" s="39"/>
+      <c r="K12" s="37"/>
       <c r="L12" s="4"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="I13" s="42"/>
-      <c r="J13" s="42"/>
-      <c r="K13" s="42"/>
+      <c r="I13" s="39"/>
+      <c r="J13" s="39"/>
+      <c r="K13" s="39"/>
     </row>
     <row r="14" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I14" s="42"/>
-      <c r="J14" s="42"/>
-      <c r="K14" s="42"/>
+      <c r="I14" s="39"/>
+      <c r="J14" s="39"/>
+      <c r="K14" s="39"/>
     </row>
     <row r="15" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D15" s="25"/>
-      <c r="E15" s="31" t="s">
+      <c r="E15" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="32"/>
-      <c r="G15" s="33"/>
-      <c r="I15" s="42"/>
-      <c r="J15" s="42"/>
-      <c r="K15" s="42"/>
+      <c r="F15" s="41"/>
+      <c r="G15" s="42"/>
+      <c r="I15" s="39"/>
+      <c r="J15" s="39"/>
+      <c r="K15" s="39"/>
     </row>
     <row r="16" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D16" s="26"/>
-      <c r="E16" s="31" t="s">
+      <c r="E16" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="F16" s="32"/>
-      <c r="G16" s="33"/>
-      <c r="I16" s="42"/>
-      <c r="J16" s="42"/>
-      <c r="K16" s="42"/>
+      <c r="F16" s="41"/>
+      <c r="G16" s="42"/>
+      <c r="I16" s="39"/>
+      <c r="J16" s="39"/>
+      <c r="K16" s="39"/>
     </row>
     <row r="17" spans="4:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D17" s="27"/>
-      <c r="E17" s="31" t="s">
+      <c r="E17" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="F17" s="32"/>
-      <c r="G17" s="33"/>
+      <c r="F17" s="41"/>
+      <c r="G17" s="42"/>
     </row>
     <row r="18" spans="4:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D18" s="24"/>
-      <c r="E18" s="31" t="s">
+      <c r="E18" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="F18" s="32"/>
-      <c r="G18" s="33"/>
+      <c r="F18" s="41"/>
+      <c r="G18" s="42"/>
     </row>
     <row r="19" spans="4:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D19" s="24"/>
-      <c r="E19" s="31" t="s">
+      <c r="E19" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="F19" s="32"/>
-      <c r="G19" s="33"/>
+      <c r="F19" s="41"/>
+      <c r="G19" s="42"/>
     </row>
     <row r="20" spans="4:18" x14ac:dyDescent="0.25">
       <c r="R20" s="22"/>

</xml_diff>

<commit_message>
add excel dated finished
</commit_message>
<xml_diff>
--- a/Experimental_data/Impurities.xlsx
+++ b/Experimental_data/Impurities.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\darshanraju\OneDrive - Delft University of Technology\Desktop\A6\Experimental_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A03B692C-1F15-47FE-AF37-A7AC01320820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A544DC56-FA94-4365-94DA-D9266E12D08D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PCP-SAFT" sheetId="1" r:id="rId1"/>
     <sheet name="KIJ_MATRIX" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
-    <sheet name="Aspen" sheetId="4" r:id="rId4"/>
+    <sheet name="Aspen" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="49">
   <si>
     <t>Molecules</t>
   </si>
@@ -62,9 +61,6 @@
     <t>No</t>
   </si>
   <si>
-    <t>Quadrupole - but fiteed with mu, sigma, epsilon</t>
-  </si>
-  <si>
     <t>Non-associating</t>
   </si>
   <si>
@@ -83,57 +79,18 @@
     <t>O2</t>
   </si>
   <si>
-    <t>H2O</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
-    <t>Strong</t>
-  </si>
-  <si>
-    <t>Secondary</t>
-  </si>
-  <si>
-    <t>Associating</t>
-  </si>
-  <si>
     <t>CO</t>
   </si>
   <si>
-    <t>Yes (small mu)</t>
-  </si>
-  <si>
     <t>Weak</t>
   </si>
   <si>
-    <t>Usually ignored -- lumped in to dispersion</t>
-  </si>
-  <si>
-    <t>NO2</t>
-  </si>
-  <si>
-    <t>Moderate</t>
-  </si>
-  <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>SO2</t>
-  </si>
-  <si>
-    <t>Polar extension with mu</t>
-  </si>
-  <si>
     <t>H2S</t>
   </si>
   <si>
-    <t>C3H8</t>
-  </si>
-  <si>
-    <t>C2H6</t>
-  </si>
-  <si>
     <t>Self pair no Kij</t>
   </si>
   <si>
@@ -143,21 +100,6 @@
     <t>No VLE data available</t>
   </si>
   <si>
-    <t>Blagoi, Y. P. Ukr. Fiz. Zh., 1960, 5, 109-114 Surface Tensions of Solutions of Liquified Gases N2-CH4 and Ar-CH4</t>
-  </si>
-  <si>
-    <t>Surface tension</t>
-  </si>
-  <si>
-    <t>Sprow, F. B.; Prausnitz, J. M. Trans. Am. Inst. Chem. Eng., 1965, 62, 1105-1111 Surfase tensions of simple liquid mixtures</t>
-  </si>
-  <si>
-    <t>https://perminc.com/resources/fundamentals-of-fluid-flow-in-porous-media/chapter-5-miscible-displacement/fluid-phase-behavior/tertiary-diagram/</t>
-  </si>
-  <si>
-    <t>TERNARY DIAGRAM BASIC</t>
-  </si>
-  <si>
     <t>Kij - polynomial</t>
   </si>
   <si>
@@ -203,12 +145,6 @@
     <t>7440-37-1</t>
   </si>
   <si>
-    <t>WATER</t>
-  </si>
-  <si>
-    <t>7732-18-5</t>
-  </si>
-  <si>
     <t>NITROGEN</t>
   </si>
   <si>
@@ -236,56 +172,23 @@
     <t>74-82-8</t>
   </si>
   <si>
-    <t>NITROGEN-DIOXIDE</t>
-  </si>
-  <si>
-    <t>10102-44-0</t>
-  </si>
-  <si>
-    <t>NITRIC-OXIDE</t>
-  </si>
-  <si>
-    <t>10102-43-9</t>
-  </si>
-  <si>
-    <t>SULFUR-DIOXIDE</t>
-  </si>
-  <si>
-    <t>O2S</t>
-  </si>
-  <si>
-    <t>SO</t>
-  </si>
-  <si>
-    <t>SULFUR-MONOXIDE-GAS</t>
-  </si>
-  <si>
-    <t>PROPANE</t>
-  </si>
-  <si>
-    <t>74-98-6</t>
-  </si>
-  <si>
-    <t>ETHANE</t>
-  </si>
-  <si>
-    <t>74-84-0</t>
-  </si>
-  <si>
-    <t>7446-09-5-</t>
-  </si>
-  <si>
-    <t>13827-32-2</t>
-  </si>
-  <si>
-    <t>yes</t>
+    <t>Quadrupole</t>
+  </si>
+  <si>
+    <t>Polar extension and association</t>
+  </si>
+  <si>
+    <t>No but there is small mu</t>
+  </si>
+  <si>
+    <t>Polar extension Ignored and lumped in to dispersion</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -316,22 +219,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -346,7 +233,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -389,14 +276,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="20">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -466,19 +347,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -645,12 +513,89 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -661,55 +606,50 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -801,15 +741,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>303610</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>5</xdr:row>
       <xdr:rowOff>59531</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>452691</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>5</xdr:row>
       <xdr:rowOff>185381</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
@@ -1191,13 +1131,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>113109</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>65485</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>238125</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>171020</xdr:rowOff>
@@ -1981,14 +1921,14 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>196453</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>160735</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>41672</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>321469</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>285751</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>147207</xdr:rowOff>
     </xdr:to>
@@ -2007,7 +1947,7 @@
           </xdr14:nvContentPartPr>
           <xdr14:nvPr macro=""/>
           <xdr14:xfrm>
-            <a:off x="7090172" y="1464469"/>
+            <a:off x="7054454" y="1464469"/>
             <a:ext cx="125016" cy="105535"/>
           </xdr14:xfrm>
         </xdr:contentPart>
@@ -2046,13 +1986,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>125016</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>53577</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>250032</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>159112</xdr:rowOff>
@@ -2073,6 +2013,136 @@
           <xdr14:nvPr macro=""/>
           <xdr14:xfrm>
             <a:off x="7018735" y="464343"/>
+            <a:ext cx="125016" cy="105535"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback xmlns="">
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="10" name="Ink 9">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5225B6B6-C1CD-4675-B722-79F91E20B070}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="5717925" y="264870"/>
+              <a:ext cx="142619" cy="123124"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>154781</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>279797</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>153160</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId25">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="24" name="Ink 23">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E31DFEBA-887C-48B5-81B1-FF9D93E4747B}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="7048500" y="1065609"/>
+            <a:ext cx="125016" cy="105535"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback xmlns="">
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="10" name="Ink 9">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5225B6B6-C1CD-4675-B722-79F91E20B070}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="5717925" y="264870"/>
+              <a:ext cx="142619" cy="123124"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>154781</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>279797</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>153160</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId26">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="25" name="Ink 24">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{19816715-B45F-43D3-8825-A9E36F20C322}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="7048500" y="863203"/>
             <a:ext cx="125016" cy="105535"/>
           </xdr14:xfrm>
         </xdr:contentPart>
@@ -2507,6 +2577,60 @@
         </inkml:channelProperties>
       </inkml:inkSource>
       <inkml:timestamp xml:id="ts0" timeString="2026-04-22T13:39:09.406"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 232 24575,'14'14'0,"-6"-5"0,1 0 0,10 7 0,-15-13 0,-3-1 0,1-1 0,0 0 0,0 1 0,0-1 0,4 1 0,-5-1 0,-1-1 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0-1 0,-1 1 0,1 0 0,-1 0 0,1-1 0,-1 1 0,1 0 0,0-1 0,-1 1 0,1-1 0,-1 1 0,1-1 0,4-5 0,5-8 0,3-3 0,53-52 0,10-13 0,-51 52-682,38-35-1,-59 60-6143</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink23.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-04-23T08:48:31.190"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 232 24575,'14'14'0,"-6"-5"0,1 0 0,10 7 0,-15-13 0,-3-1 0,1-1 0,0 0 0,0 1 0,0-1 0,4 1 0,-5-1 0,-1-1 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0-1 0,-1 1 0,1 0 0,-1 0 0,1-1 0,-1 1 0,1 0 0,0-1 0,-1 1 0,1-1 0,-1 1 0,1-1 0,4-5 0,5-8 0,3-3 0,53-52 0,10-13 0,-51 52-682,38-35-1,-59 60-6143</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink24.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-04-23T08:48:32.518"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
       <inkml:brushProperty name="width" value="0.05" units="cm"/>
@@ -3028,13 +3152,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.75" customWidth="1"/>
+    <col min="2" max="2" width="26.25" customWidth="1"/>
     <col min="3" max="3" width="17.25" customWidth="1"/>
     <col min="4" max="4" width="44.5" customWidth="1"/>
-    <col min="5" max="5" width="40.125" customWidth="1"/>
+    <col min="5" max="5" width="49.25" customWidth="1"/>
     <col min="6" max="6" width="24.375" customWidth="1"/>
     <col min="7" max="7" width="21.125" customWidth="1"/>
   </cols>
@@ -3071,10 +3195,10 @@
         <v>7</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>8</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>9</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>7</v>
@@ -3082,7 +3206,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>7</v>
@@ -3094,7 +3218,7 @@
         <v>7</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>7</v>
@@ -3102,7 +3226,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>7</v>
@@ -3114,7 +3238,7 @@
         <v>7</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>7</v>
@@ -3122,7 +3246,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>7</v>
@@ -3131,10 +3255,10 @@
         <v>7</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>7</v>
@@ -3142,7 +3266,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>7</v>
@@ -3154,7 +3278,7 @@
         <v>7</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>7</v>
@@ -3162,7 +3286,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>7</v>
@@ -3174,7 +3298,7 @@
         <v>7</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>7</v>
@@ -3185,165 +3309,45 @@
         <v>15</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="E8" s="3" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F15" s="3" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:F7 A10:F15 B8:C8 E8:F8 A9 C9:F9" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:F1 A9:B9 A8 C8 A3:F4 A2:C2 E2:F2 F8 A6:F7 A5:C5 E5:F5 D9 F9" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3358,46 +3362,37 @@
     <col min="17" max="17" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="14" t="s">
         <v>6</v>
       </c>
       <c r="C1" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="E1" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="F1" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="G1" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="10" t="s">
-        <v>14</v>
-      </c>
       <c r="H1" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="I1" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="J1" s="32" t="s">
-        <v>26</v>
-      </c>
-      <c r="K1" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="13" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" s="30" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="7"/>
@@ -3407,46 +3402,35 @@
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
-      <c r="I2" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="J2" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="K2" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="L2" s="5"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
-        <v>10</v>
+      <c r="I2" s="31"/>
+    </row>
+    <row r="3" spans="1:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="17" t="s">
+        <v>9</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="12"/>
       <c r="D3" s="6"/>
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
-      <c r="G3" s="14">
+      <c r="G3" s="13">
         <v>0</v>
       </c>
       <c r="H3" s="5"/>
-      <c r="I3" s="34">
-        <v>0</v>
-      </c>
-      <c r="J3" s="34">
-        <v>0</v>
-      </c>
-      <c r="K3" s="34">
-        <v>0</v>
-      </c>
-      <c r="L3" s="6"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="20"/>
+      <c r="I3" s="32"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="M3" s="28"/>
+      <c r="N3" s="29"/>
+    </row>
+    <row r="4" spans="1:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="33"/>
+      <c r="C4" s="34"/>
       <c r="D4" s="4"/>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
@@ -3455,246 +3439,168 @@
       <c r="I4" s="35">
         <v>0</v>
       </c>
-      <c r="J4" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="K4" s="35">
-        <v>0</v>
-      </c>
-      <c r="L4" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="20"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="M4" s="28"/>
+      <c r="N4" s="29"/>
+    </row>
+    <row r="5" spans="1:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="33"/>
+      <c r="C5" s="34"/>
       <c r="D5" s="8"/>
       <c r="E5" s="7"/>
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
-      <c r="I5" s="35">
-        <v>0</v>
-      </c>
-      <c r="J5" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="K5" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="20"/>
+      <c r="I5" s="31"/>
+      <c r="K5" s="23"/>
+      <c r="L5" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="M5" s="28"/>
+      <c r="N5" s="29"/>
+    </row>
+    <row r="6" spans="1:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="33"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="33"/>
       <c r="E6" s="8"/>
       <c r="F6" s="7"/>
-      <c r="G6" s="14">
+      <c r="G6" s="13">
         <v>0</v>
       </c>
       <c r="H6" s="5"/>
-      <c r="I6" s="35">
-        <v>0</v>
-      </c>
-      <c r="J6" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="K6" s="33">
-        <v>0</v>
-      </c>
-      <c r="L6" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="20"/>
+      <c r="I6" s="31"/>
+      <c r="K6" s="20"/>
+      <c r="L6" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="M6" s="28"/>
+      <c r="N6" s="29"/>
+    </row>
+    <row r="7" spans="1:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="33"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
       <c r="F7" s="8"/>
       <c r="G7" s="4"/>
-      <c r="H7" s="14">
+      <c r="H7" s="13">
         <v>0</v>
       </c>
       <c r="I7" s="35">
         <v>0</v>
       </c>
-      <c r="J7" s="35">
-        <v>0</v>
-      </c>
-      <c r="K7" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="L7" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="20"/>
+      <c r="K7" s="20"/>
+      <c r="L7" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="M7" s="28"/>
+      <c r="N7" s="29"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="33"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
       <c r="H8" s="7"/>
-      <c r="I8" s="35">
-        <v>0</v>
-      </c>
-      <c r="J8" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="K8" s="33"/>
-      <c r="L8" s="43"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="H9" s="8"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="35">
-        <v>0</v>
-      </c>
-      <c r="K9" s="35">
-        <v>0</v>
-      </c>
-      <c r="L9" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="I10" s="37"/>
-      <c r="J10" s="38"/>
-      <c r="K10" s="35" t="s">
-        <v>80</v>
-      </c>
-      <c r="L10" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="I11" s="39"/>
-      <c r="J11" s="37"/>
-      <c r="K11" s="38"/>
-      <c r="L11" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="I12" s="39"/>
-      <c r="J12" s="39"/>
-      <c r="K12" s="37"/>
-      <c r="L12" s="4"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="I13" s="39"/>
-      <c r="J13" s="39"/>
-      <c r="K13" s="39"/>
-    </row>
-    <row r="14" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I14" s="39"/>
-      <c r="J14" s="39"/>
-      <c r="K14" s="39"/>
-    </row>
-    <row r="15" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D15" s="25"/>
-      <c r="E15" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="F15" s="41"/>
-      <c r="G15" s="42"/>
-      <c r="I15" s="39"/>
-      <c r="J15" s="39"/>
-      <c r="K15" s="39"/>
-    </row>
-    <row r="16" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D16" s="26"/>
-      <c r="E16" s="40" t="s">
-        <v>33</v>
-      </c>
-      <c r="F16" s="41"/>
-      <c r="G16" s="42"/>
-      <c r="I16" s="39"/>
-      <c r="J16" s="39"/>
-      <c r="K16" s="39"/>
-    </row>
-    <row r="17" spans="4:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D17" s="27"/>
-      <c r="E17" s="40" t="s">
-        <v>34</v>
-      </c>
-      <c r="F17" s="41"/>
-      <c r="G17" s="42"/>
-    </row>
-    <row r="18" spans="4:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D18" s="24"/>
-      <c r="E18" s="40" t="s">
-        <v>40</v>
-      </c>
-      <c r="F18" s="41"/>
-      <c r="G18" s="42"/>
-    </row>
-    <row r="19" spans="4:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D19" s="24"/>
-      <c r="E19" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="F19" s="41"/>
-      <c r="G19" s="42"/>
-    </row>
-    <row r="20" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R20" s="22"/>
-    </row>
-    <row r="21" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R21" s="23"/>
-    </row>
-    <row r="22" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R22" s="23"/>
-    </row>
-    <row r="23" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R23" s="23"/>
-    </row>
-    <row r="24" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R24" s="23"/>
-    </row>
-    <row r="25" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R25" s="23"/>
-    </row>
-    <row r="26" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R26" s="23"/>
-    </row>
-    <row r="27" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R27" s="23"/>
-    </row>
-    <row r="28" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R28" s="23"/>
-    </row>
-    <row r="29" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R29" s="23"/>
-    </row>
-    <row r="30" spans="4:18" x14ac:dyDescent="0.25">
-      <c r="R30" s="23"/>
+      <c r="I8" s="36"/>
+    </row>
+    <row r="9" spans="1:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="38"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="38"/>
+      <c r="G9" s="38"/>
+      <c r="H9" s="38"/>
+      <c r="I9" s="39"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I10" s="26"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I11" s="26"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I12" s="26"/>
+      <c r="J12" s="26"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I13" s="26"/>
+      <c r="J13" s="26"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J14" s="26"/>
+      <c r="K14" s="26"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J15" s="26"/>
+      <c r="K15" s="26"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J16" s="26"/>
+      <c r="K16" s="26"/>
+    </row>
+    <row r="20" spans="18:18" x14ac:dyDescent="0.25">
+      <c r="R20" s="18"/>
+    </row>
+    <row r="21" spans="18:18" x14ac:dyDescent="0.25">
+      <c r="R21" s="19"/>
+    </row>
+    <row r="22" spans="18:18" x14ac:dyDescent="0.25">
+      <c r="R22" s="19"/>
+    </row>
+    <row r="23" spans="18:18" x14ac:dyDescent="0.25">
+      <c r="R23" s="19"/>
+    </row>
+    <row r="24" spans="18:18" x14ac:dyDescent="0.25">
+      <c r="R24" s="19"/>
+    </row>
+    <row r="25" spans="18:18" x14ac:dyDescent="0.25">
+      <c r="R25" s="19"/>
+    </row>
+    <row r="26" spans="18:18" x14ac:dyDescent="0.25">
+      <c r="R26" s="19"/>
+    </row>
+    <row r="27" spans="18:18" x14ac:dyDescent="0.25">
+      <c r="R27" s="19"/>
+    </row>
+    <row r="28" spans="18:18" x14ac:dyDescent="0.25">
+      <c r="R28" s="19"/>
+    </row>
+    <row r="29" spans="18:18" x14ac:dyDescent="0.25">
+      <c r="R29" s="19"/>
+    </row>
+    <row r="30" spans="18:18" x14ac:dyDescent="0.25">
+      <c r="R30" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="L7:N7"/>
+    <mergeCell ref="L6:N6"/>
+    <mergeCell ref="L5:N5"/>
+    <mergeCell ref="L4:N4"/>
+    <mergeCell ref="L3:N3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -3703,49 +3609,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA83B7F6-A1DD-4E6A-A85F-87A5C7B53BBB}">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="101.375" customWidth="1"/>
-    <col min="2" max="2" width="17.625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="21" t="s">
-        <v>38</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A7" r:id="rId1" xr:uid="{65146813-479E-4790-8DA9-6A94B40E8577}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AF32340-A001-4725-A15E-F63437E1FB43}">
   <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -3756,19 +3619,19 @@
   <sheetData>
     <row r="1" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -3776,265 +3639,147 @@
         <v>6</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>56</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>62</v>
+        <v>17</v>
+      </c>
+      <c r="E8" s="25">
+        <v>2148878</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="29">
-        <v>2148878</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="E13" s="30" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="H18" s="28"/>
+        <v>12</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" spans="8:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H18" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Except CO2 and H2 pairs all are updated
</commit_message>
<xml_diff>
--- a/Experimental_data/Impurities.xlsx
+++ b/Experimental_data/Impurities.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\darshanraju\OneDrive - Delft University of Technology\Desktop\A6\Experimental_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A544DC56-FA94-4365-94DA-D9266E12D08D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B316DC63-2E3F-4E8E-936A-B9F9159F640C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PCP-SAFT" sheetId="1" r:id="rId1"/>

</xml_diff>